<commit_message>
Atualização na votação interativa e uma nova tela do windows forms para ver os votos
</commit_message>
<xml_diff>
--- a/candidatos.xlsx
+++ b/candidatos.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <x:fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29518"/>
+  <x:fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29525"/>
   <x:workbookPr codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B145DA0-74BF-4448-823E-17F6147B14B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{11B2EF4F-0BD8-4330-AC0B-0BCB2CE17410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <x:bookViews>
     <x:workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="0" activeTab="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </x:bookViews>
@@ -55,43 +55,46 @@
     <x:t>1</x:t>
   </x:si>
   <x:si>
-    <x:t>123</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Vitor</x:t>
-  </x:si>
-  <x:si>
-    <x:t>vitin</x:t>
-  </x:si>
-  <x:si>
-    <x:t>qe</x:t>
+    <x:t>4578</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ana Clara</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Clarinha</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PT</x:t>
   </x:si>
   <x:si>
     <x:t>2</x:t>
   </x:si>
   <x:si>
-    <x:t>4512</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Cleytinho</x:t>
-  </x:si>
-  <x:si>
-    <x:t>clay</x:t>
-  </x:si>
-  <x:si>
-    <x:t>er</x:t>
+    <x:t>447</x:t>
+  </x:si>
+  <x:si>
+    <x:t>João Vitor</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Vitinho</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PRESSOL</x:t>
   </x:si>
   <x:si>
     <x:t>3</x:t>
   </x:si>
   <x:si>
-    <x:t>5555</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ada</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ad</x:t>
+    <x:t>5874</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Matheus</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Matheusin</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Aladin</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -519,7 +522,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="F2" s="0">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -556,10 +559,10 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Forms do resultado finalizado, votação interativa foi corrigida, e agora toda vez que o sistema se inicializar o excel irá ser formatado para que toda vez que o sistema abrir simular uma nova votação
</commit_message>
<xml_diff>
--- a/candidatos.xlsx
+++ b/candidatos.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <x:fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29525"/>
+  <x:fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
   <x:workbookPr codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{11B2EF4F-0BD8-4330-AC0B-0BCB2CE17410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A433DEC-F8E5-4F6C-8461-8C461D1EE980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <x:bookViews>
     <x:workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="0" activeTab="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </x:bookViews>
@@ -52,10 +52,13 @@
     <x:t>VOTOS</x:t>
   </x:si>
   <x:si>
+    <x:t>0</x:t>
+  </x:si>
+  <x:si>
     <x:t>1</x:t>
   </x:si>
   <x:si>
-    <x:t>4578</x:t>
+    <x:t>5555</x:t>
   </x:si>
   <x:si>
     <x:t>Ana Clara</x:t>
@@ -70,31 +73,16 @@
     <x:t>2</x:t>
   </x:si>
   <x:si>
-    <x:t>447</x:t>
+    <x:t>4444</x:t>
   </x:si>
   <x:si>
     <x:t>João Vitor</x:t>
   </x:si>
   <x:si>
-    <x:t>Vitinho</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PRESSOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5874</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Matheus</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Matheusin</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Aladin</x:t>
+    <x:t>Vitin</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PESSOL</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -478,14 +466,14 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F1"/>
+  <x:dimension ref="A1:I1"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="2" width="9.090625" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="16.570312" style="0" bestFit="1" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:6">
+    <x:row r="1" spans="1:9">
       <x:c r="A1" s="0" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -504,65 +492,51 @@
       <x:c r="F1" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="H1" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I1" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
-    <x:row r="2" spans="1:6">
+    <x:row r="2" spans="1:9">
       <x:c r="A2" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F2" s="0" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B2" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C2" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D2" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E2" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F2" s="0">
-        <x:v>4</x:v>
-      </x:c>
     </x:row>
-    <x:row r="3" spans="1:6">
+    <x:row r="3" spans="1:9">
       <x:c r="A3" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F3" s="0">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:6">
-      <x:c r="A4" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="D4" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="E4" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="F4" s="0">
-        <x:v>1</x:v>
+      <x:c r="F3" s="0" t="s">
+        <x:v>6</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Finalizei alguns detalhes e corrigi algumas falhas
</commit_message>
<xml_diff>
--- a/candidatos.xlsx
+++ b/candidatos.xlsx
@@ -52,37 +52,52 @@
     <x:t>VOTOS</x:t>
   </x:si>
   <x:si>
-    <x:t>0</x:t>
+    <x:t>2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4</x:t>
   </x:si>
   <x:si>
     <x:t>1</x:t>
   </x:si>
   <x:si>
+    <x:t>666</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ana Gonçalves</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Aninha Favelada</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PT</x:t>
+  </x:si>
+  <x:si>
     <x:t>5555</x:t>
   </x:si>
   <x:si>
-    <x:t>Ana Clara</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Clarinha</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4444</x:t>
-  </x:si>
-  <x:si>
-    <x:t>João Vitor</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Vitin</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PESSOL</x:t>
+    <x:t>Flavio Machado</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Flávin do Pneu</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PV</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12345</x:t>
+  </x:si>
+  <x:si>
+    <x:t>João Vitor Cabral</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Jãozin do grau</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PH</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -496,32 +511,32 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="I1" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:9">
       <x:c r="A2" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="F2" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F2" s="0">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:9">
       <x:c r="A3" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>13</x:v>
@@ -535,7 +550,27 @@
       <x:c r="E3" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="F3" s="0" t="s">
+      <x:c r="F3" s="0">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:9">
+      <x:c r="A4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="F4" s="0">
         <x:v>6</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Alterando a tela de Votacao Interativa para apresentar como votar nulo e como votar em branco
</commit_message>
<xml_diff>
--- a/candidatos.xlsx
+++ b/candidatos.xlsx
@@ -98,6 +98,18 @@
   </x:si>
   <x:si>
     <x:t>PH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>111</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Jeferson</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Jefercinho</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LL</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -531,7 +543,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="F2" s="0">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:9">
@@ -572,6 +584,26 @@
       </x:c>
       <x:c r="F4" s="0">
         <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:9">
+      <x:c r="A5" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F5" s="0">
+        <x:v>2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>